<commit_message>
Scrape PDPC's redesigned site without a browser, and refresh the data
</commit_message>
<xml_diff>
--- a/pdpc_analysis.xlsx
+++ b/pdpc_analysis.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yearly Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Penalty Distribution" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Obligation Mix" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Outcomes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notable Cases" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Yearly Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Penalty Distribution" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Obligation Mix" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Decision Outcomes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Notable Cases" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -573,25 +573,25 @@
         <v>2016</v>
       </c>
       <c r="B3" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>104000</v>
+        <v>109000</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>13000</v>
+        <v>12111</v>
       </c>
       <c r="G3" s="5" t="n">
         <v>50000</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -617,7 +617,7 @@
         <v>18000</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -643,7 +643,7 @@
         <v>30000</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -680,16 +680,16 @@
         <v>45</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>420500</v>
+        <v>413000</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>16820</v>
+        <v>17208</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>120000</v>
@@ -703,13 +703,13 @@
         <v>2021</v>
       </c>
       <c r="B8" s="7" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>15</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E8" s="8" t="n">
         <v>309000</v>
@@ -721,7 +721,7 @@
         <v>74000</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
@@ -755,13 +755,13 @@
         <v>2023</v>
       </c>
       <c r="B10" s="7" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10" s="7" t="n">
         <v>9</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10" s="8" t="n">
         <v>343800</v>
@@ -773,7 +773,7 @@
         <v>82000</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11">
@@ -781,19 +781,19 @@
         <v>2024</v>
       </c>
       <c r="B11" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="C11" s="4" t="n">
         <v>12</v>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>11</v>
       </c>
       <c r="D11" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>357000</v>
+        <v>431000</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>32454</v>
+        <v>35916</v>
       </c>
       <c r="G11" s="5" t="n">
         <v>120000</v>
@@ -833,13 +833,13 @@
         <v>2026</v>
       </c>
       <c r="B13" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C13" s="4" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" s="5" t="n">
         <v>148750</v>
@@ -861,25 +861,25 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>3498050</v>
+        <v>3569550</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>25165</v>
+        <v>25496</v>
       </c>
       <c r="G14" s="10" t="n">
         <v>315000</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -938,7 +938,7 @@
         <v>69</v>
       </c>
       <c r="C3" s="12" t="n">
-        <v>0.4964028776978417</v>
+        <v>0.4928571428571429</v>
       </c>
     </row>
     <row r="4">
@@ -951,7 +951,7 @@
         <v>51</v>
       </c>
       <c r="C4" s="14" t="n">
-        <v>0.3669064748201439</v>
+        <v>0.3642857142857143</v>
       </c>
     </row>
     <row r="5">
@@ -961,10 +961,10 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>0.1079136690647482</v>
+        <v>0.1142857142857143</v>
       </c>
     </row>
     <row r="6">
@@ -977,7 +977,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="14" t="n">
-        <v>0.02877697841726619</v>
+        <v>0.02857142857142857</v>
       </c>
     </row>
     <row r="7">
@@ -1007,7 +1007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1052,13 +1052,13 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="C3" s="12" t="n">
-        <v>0.8151658767772512</v>
+        <v>0.8472222222222222</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>24437</v>
+        <v>25674</v>
       </c>
     </row>
     <row r="4">
@@ -1068,29 +1068,29 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C4" s="14" t="n">
-        <v>0.08056872037914692</v>
+        <v>0.09722222222222222</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>18791</v>
+        <v>27269</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>Accountability, Protection</t>
+          <t>Protection, Openness</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>0.03791469194312796</v>
+        <v>0.01851851851851852</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>26100</v>
+        <v>30333</v>
       </c>
     </row>
     <row r="6">
@@ -1100,58 +1100,58 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C6" s="14" t="n">
-        <v>0.01895734597156398</v>
+        <v>0.01388888888888889</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>19250</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>Protection, Protection</t>
+          <t>Protection, Accountability, Retention Limitation</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>0.01421800947867299</v>
+        <v>0.004629629629629629</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>92666</v>
+        <v>37500</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>Protection, Consent</t>
+          <t>Protection, Openness, Transfer Limitation</t>
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C8" s="14" t="n">
-        <v>0.009478672985781991</v>
+        <v>0.004629629629629629</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>7000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>Protection, Transfer Limitation</t>
+          <t>Protection, Purpose Limitation</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>0.004739336492890996</v>
+        <v>0.004629629629629629</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>0</v>
@@ -1160,65 +1160,33 @@
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>Protection, Accountability, Retention Limitation</t>
+          <t>Protection, Transfer Limitation</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="14" t="n">
-        <v>0.004739336492890996</v>
+        <v>0.004629629629629629</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>37500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>Protection, Retention Limitation, Accountability</t>
+          <t>Protection, Consent</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="12" t="n">
-        <v>0.004739336492890996</v>
+        <v>0.004629629629629629</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>Protection, Accountability, Transfer Limitation</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="14" t="n">
-        <v>0.004739336492890996</v>
-      </c>
-      <c r="D12" s="8" t="n">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>Protection, Purpose Limitation</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" s="12" t="n">
-        <v>0.004739336492890996</v>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>0</v>
+        <v>7000</v>
       </c>
     </row>
   </sheetData>
@@ -1274,10 +1242,10 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C3" s="12" t="n">
-        <v>0.1469194312796208</v>
+        <v>0.1666666666666667</v>
       </c>
     </row>
     <row r="4">
@@ -1287,10 +1255,10 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C4" s="14" t="n">
-        <v>0.5118483412322274</v>
+        <v>0.4814814814814815</v>
       </c>
     </row>
     <row r="5">
@@ -1300,10 +1268,10 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>0.1137440758293839</v>
+        <v>0.1064814814814815</v>
       </c>
     </row>
     <row r="6">
@@ -1316,7 +1284,7 @@
         <v>39</v>
       </c>
       <c r="C6" s="14" t="n">
-        <v>0.1848341232227488</v>
+        <v>0.1805555555555556</v>
       </c>
     </row>
     <row r="7">
@@ -1326,10 +1294,10 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>0.04265402843601896</v>
+        <v>0.04629629629629629</v>
       </c>
     </row>
     <row r="8">
@@ -1339,10 +1307,10 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C8" s="14" t="n">
-        <v>0</v>
+        <v>0.01851851851851852</v>
       </c>
     </row>
   </sheetData>
@@ -1440,12 +1408,12 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>Re Keppel Telecommunications &amp; Transportation</t>
+          <t>Re Secur Solutions Group</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>02 Aug 2024</t>
+          <t>24 Nov 2020</t>
         </is>
       </c>
       <c r="C5" s="10" t="n">
@@ -1453,19 +1421,19 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>[2024] SGPDPC 3</t>
+          <t>[2020] SGPDPC 8</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Re Secur Solutions Group</t>
+          <t>Re Keppel Telecommunications &amp; Transportation</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>24 Nov 2020</t>
+          <t>02 Aug 2024</t>
         </is>
       </c>
       <c r="C6" s="17" t="n">
@@ -1473,7 +1441,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>[2020] SGPDPC 8</t>
+          <t>[2024] SGPDPC 3</t>
         </is>
       </c>
     </row>
@@ -1580,20 +1548,20 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>Re RedMart</t>
+          <t>Re PPLingo</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>19 Dec 2022</t>
+          <t>21 Mar 2024</t>
         </is>
       </c>
       <c r="C12" s="17" t="n">
-        <v>72000</v>
+        <v>74000</v>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>[2022] SGPDPC 8</t>
+          <t>[2023] SGPDPC 12</t>
         </is>
       </c>
     </row>

</xml_diff>